<commit_message>
[auto-snapshot] 2026-04-28 16:00 | onda-hompage | 25 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/강화군_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/강화군_네일샵.xlsx
@@ -564,29 +564,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>그레이스네일</t>
+          <t>프프네일</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>lumirode@naver.com</t>
+          <t>daonnail0305@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1379-5084</t>
+          <t>0507-1407-8841</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로248번길 24 갑룡프라자 2층</t>
+          <t>인천광역시 강화군 강화읍 남문안길 5-1 1층</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/grace_nail_?igsh=eGhhYXZlaGl0Z3hh&amp;utm_source=qr</t>
+          <t>https://www.instagram.com/ff__nail</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>159</v>
+        <v>5</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R2" t="n">
-        <v>160</v>
+        <v>7</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,17 +636,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1030374689</t>
+          <t>1170338521</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1030374689</t>
+          <t>https://m.place.naver.com/place/1170338521</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -658,29 +658,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>달빛네일</t>
+          <t>오니네일</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>duoshan_sz@naver.com</t>
+          <t>wjsska1907@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1316-8875</t>
+          <t>0507-1311-0663</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 310 201호 달빛네일</t>
+          <t>인천광역시 강화군 강화읍 갑룡길 29 1층, 카페88 내부위치</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://open.kakao.com/o/sLs1Sagi</t>
+          <t>http://instagram.com/oninail_</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -706,7 +706,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,17 +730,17 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2052753261</t>
+          <t>1245994155</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2052753261</t>
+          <t>https://m.place.naver.com/place/1245994155</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -752,34 +752,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>미뇽네일</t>
+          <t>지니네일</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>akstjd1018@naver.com</t>
+          <t>goto_seoul@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1381-9702</t>
+          <t>0507-1316-6480</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 347-1 101호</t>
+          <t>인천광역시 강화군 강화읍 남문안길32번길 8 2층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>http://pf.kakao.com/_hkxiqG</t>
+          <t>http://www.instagram.com/jineenail</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -800,7 +800,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>125</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
         <v>3</v>
       </c>
       <c r="R4" t="n">
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,17 +824,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1280952259</t>
+          <t>1155579596</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1280952259</t>
+          <t>https://m.place.naver.com/place/1155579596</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -846,30 +846,34 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>제이네일</t>
+          <t>미뇽네일</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>rhkdmswl@naver.com</t>
+          <t>akstjd1018@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0507-1381-9702</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 향나무길28번길 13-1</t>
+          <t>인천광역시 강화군 강화읍 강화대로 347-1 101호</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/j.nail_shop</t>
+          <t>http://pf.kakao.com/_hkxiqG</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -890,7 +894,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -899,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>125</v>
       </c>
       <c r="Q5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>128</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -914,17 +918,17 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1237271418</t>
+          <t>1280952259</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1237271418</t>
+          <t>https://m.place.naver.com/place/1280952259</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -936,29 +940,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>퍼플리네일</t>
+          <t>코코로네일</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>u_un0709@naver.com</t>
+          <t>romina97@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0507-1315-4140</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 선원면 중앙로 162-3 2층</t>
+          <t>인천광역시 강화군 길상면 온수길 46</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/purply._.nail/</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -989,17 +989,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="n">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1008,17 +1008,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2094549338</t>
+          <t>1049963433</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2094549338</t>
+          <t>https://m.place.naver.com/place/1049963433</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1120,29 +1120,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>뉴얼리네일</t>
+          <t>이뽐뷰티 강화점</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kimaechin01@naver.com</t>
+          <t>leebbom_kh@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0507-1429-1729</t>
+          <t>0507-1385-2307</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 선원면 중앙로 162-31 서희스타힐스 106동 1층 상가</t>
+          <t>인천광역시 강화군 강화읍 동문안길 7 B동 101호</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/nurely_nail</t>
+          <t>https://blog.naver.com/leebbom_kh</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>26</v>
+        <v>101</v>
       </c>
       <c r="Q8" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="R8" t="n">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1192,17 +1192,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2009541921</t>
+          <t>1404657024</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2009541921</t>
+          <t>https://m.place.naver.com/place/1404657024</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1214,29 +1214,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>레푸스 강화점</t>
+          <t>뉴얼리네일</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>refuss_ganghwa@naver.com</t>
+          <t>kimaechin01@naver.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0507-1409-2278</t>
+          <t>0507-1429-1729</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 충렬사로 25 남산빌딩 2층 202호</t>
+          <t>인천광역시 강화군 선원면 중앙로 162-31 서희스타힐스 106동 1층 상가</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@강화레푸스</t>
+          <t>https://www.instagram.com/nurely_nail</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1271,13 +1271,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R9" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1286,17 +1286,17 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1506333714</t>
+          <t>2009541921</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1506333714</t>
+          <t>https://m.place.naver.com/place/2009541921</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1308,29 +1308,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>루비네일</t>
+          <t>비너스네일앤뷰티</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ruby1004_mj@naver.com</t>
+          <t>hankyuldata@naver.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0507-1342-4252</t>
+          <t>0507-1309-4148</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 중앙로 68 하나로마트 2층 214호</t>
+          <t>인천광역시 강화군 강화읍 신문길 42 2층</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/venus_nail4148</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1361,17 +1361,17 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1380,17 +1380,17 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1791159276</t>
+          <t>1141156599</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1791159276</t>
+          <t>https://m.place.naver.com/place/1141156599</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1402,25 +1402,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>온리원네일</t>
+          <t>그레이스네일</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>nail_one@naver.com</t>
+          <t>lumirode@naver.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0507-1379-5084</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로248번길 28-4 1층 102호</t>
+          <t>인천광역시 강화군 강화읍 강화대로248번길 24 갑룡프라자 2층</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/__only_one__nail</t>
+          <t>https://www.instagram.com/grace_nail_?igsh=eGhhYXZlaGl0Z3hh&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1455,13 +1459,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>1</v>
+        <v>159</v>
       </c>
       <c r="Q11" t="n">
         <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>2</v>
+        <v>160</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1470,17 +1474,17 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2039624196</t>
+          <t>1030374689</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2039624196</t>
+          <t>https://m.place.naver.com/place/1030374689</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1492,25 +1496,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>코코로네일</t>
+          <t>소소네일</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>romina97@naver.com</t>
+          <t>iamkimz@naver.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0507-1327-9628</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 길상면 온수길 46</t>
+          <t>인천광역시 강화군 강화읍 강화대로404번길 9 2층 윈썸헤어&amp;소소네일</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/sosonail_y?igsh=djM3NzVmbHM5eDRo&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1520,7 +1528,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1541,17 +1549,17 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
         <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1560,17 +1568,17 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1049963433</t>
+          <t>1958174820</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1049963433</t>
+          <t>https://m.place.naver.com/place/1958174820</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1582,29 +1590,25 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>소소네일</t>
+          <t>무</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>iamkimz@naver.com</t>
+          <t>sooks_room@naver.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>0507-1327-9628</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로404번길 9 2층 윈썸헤어&amp;소소네일</t>
+          <t>인천광역시 강화군 강화읍 강화대로 394</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/sosonail_y?igsh=djM3NzVmbHM5eDRo&amp;utm_source=qr</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1614,7 +1618,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1635,17 +1639,17 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R13" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1654,17 +1658,17 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1958174820</t>
+          <t>36721147</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958174820</t>
+          <t>https://m.place.naver.com/place/36721147</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1676,25 +1680,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>비너스네일앤뷰티</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>루비네일</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ruby1004_mj@naver.com</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0507-1309-4148</t>
+          <t>0507-1342-4252</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 신문길 42 2층</t>
+          <t>인천광역시 강화군 강화읍 중앙로 68 하나로마트 2층 214호</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/venus_nail4148</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1704,7 +1712,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1725,17 +1733,17 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1744,17 +1752,17 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1141156599</t>
+          <t>1791159276</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1141156599</t>
+          <t>https://m.place.naver.com/place/1791159276</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1766,29 +1774,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>프프네일</t>
+          <t>리네일아트 강화점</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>to_nail@naver.com</t>
+          <t>sg20092@naver.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0507-1407-8841</t>
+          <t>0507-1416-0155</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 남문안길 5-1 1층</t>
+          <t>인천광역시 강화군 강화읍 갑룡길 33-1</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/ff__nail</t>
+          <t>https://blog.naver.com/sg20092</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1803,7 +1811,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1819,17 +1827,17 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1838,17 +1846,17 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1170338521</t>
+          <t>1180020313</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1170338521</t>
+          <t>https://m.place.naver.com/place/1180020313</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1860,29 +1868,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>이뽐뷰티 강화점</t>
+          <t>네일홀릭</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>leebbom_kh@naver.com</t>
+          <t>minmin0319@naver.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0507-1385-2307</t>
+          <t>0507-1480-4549</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 동문안길 7 B동 101호</t>
+          <t>인천광역시 강화군 강화읍 강화대로 421 2층네일홀릭</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/leebbom_kh</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1892,12 +1900,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1913,17 +1921,17 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>101</v>
+        <v>7</v>
       </c>
       <c r="Q16" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>115</v>
+        <v>7</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1932,17 +1940,17 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1404657024</t>
+          <t>1716746742</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1404657024</t>
+          <t>https://m.place.naver.com/place/1716746742</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -1954,29 +1962,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>네일홀릭</t>
+          <t>퍼플리네일</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>minmin0319@naver.com</t>
+          <t>u_un0709@naver.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0507-1480-4549</t>
+          <t>0507-1315-4140</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 421 2층네일홀릭</t>
+          <t>인천광역시 강화군 선원면 중앙로 162-3 2층</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/purply._.nail/</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1986,7 +1994,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2007,17 +2015,17 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2026,17 +2034,17 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1716746742</t>
+          <t>2094549338</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1716746742</t>
+          <t>https://m.place.naver.com/place/2094549338</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -2048,29 +2056,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>리네일아트 강화점</t>
+          <t>온리원네일</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sg20092@naver.com</t>
+          <t>nail_one@naver.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>0507-1416-0155</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 갑룡길 33-1</t>
+          <t>인천광역시 강화군 강화읍 강화대로248번길 28-4 1층 102호</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/sg20092</t>
+          <t>https://www.instagram.com/__only_one__nail</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2085,7 +2089,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2101,17 +2105,17 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2120,17 +2124,17 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1180020313</t>
+          <t>2039624196</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1180020313</t>
+          <t>https://m.place.naver.com/place/2039624196</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -2142,29 +2146,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>오니네일</t>
+          <t>레푸스 강화점</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>wjsska1907@naver.com</t>
+          <t>refuss_ganghwa@naver.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0507-1311-0663</t>
+          <t>0507-1409-2278</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 갑룡길 29 1층, 카페88 내부위치</t>
+          <t>인천광역시 강화군 강화읍 충렬사로 25 남산빌딩 2층 202호</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>http://instagram.com/oninail_</t>
+          <t>https://www.youtube.com/@강화레푸스</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2179,7 +2183,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2199,13 +2203,13 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="Q19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2214,17 +2218,17 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1245994155</t>
+          <t>1506333714</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1245994155</t>
+          <t>https://m.place.naver.com/place/1506333714</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -2236,29 +2240,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>지니네일</t>
+          <t>제이네일</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>goto_seoul@naver.com</t>
+          <t>morningapple6@naver.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>0507-1316-6480</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 남문안길32번길 8 2층</t>
+          <t>인천광역시 강화군 강화읍 향나무길28번길 13-1</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>http://www.instagram.com/jineenail</t>
+          <t>https://www.instagram.com/j.nail_shop</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2293,13 +2293,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2308,17 +2308,17 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1155579596</t>
+          <t>1237271418</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1155579596</t>
+          <t>https://m.place.naver.com/place/1237271418</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -2330,21 +2330,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>무</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>달빛네일</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>duoshan_sz@naver.com</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0507-1316-8875</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 394</t>
+          <t>인천광역시 강화군 강화읍 강화대로 310 201호 달빛네일</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://open.kakao.com/o/sLs1Sagi</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2354,7 +2362,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2370,22 +2378,22 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2394,17 +2402,17 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>36721147</t>
+          <t>2052753261</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/36721147</t>
+          <t>https://m.place.naver.com/place/2052753261</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-30 12:00 | onda-hompage | 87 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/강화군_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/강화군_네일샵.xlsx
@@ -564,29 +564,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>프프네일</t>
+          <t>리네일아트 강화점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>daonnail0305@naver.com</t>
+          <t>sg20092@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1407-8841</t>
+          <t>0507-1416-0155</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 남문안길 5-1 1층</t>
+          <t>인천광역시 강화군 강화읍 갑룡길 33-1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/ff__nail</t>
+          <t>https://blog.naver.com/sg20092</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -617,17 +617,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -636,17 +636,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1170338521</t>
+          <t>1180020313</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1170338521</t>
+          <t>https://m.place.naver.com/place/1180020313</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -658,29 +658,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>오니네일</t>
+          <t>코코로네일</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>wjsska1907@naver.com</t>
+          <t>romina97@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0507-1311-0663</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 갑룡길 29 1층, 카페88 내부위치</t>
+          <t>인천광역시 강화군 길상면 온수길 46</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>http://instagram.com/oninail_</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -690,7 +686,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -711,17 +707,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="Q3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,17 +726,17 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1245994155</t>
+          <t>1049963433</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1245994155</t>
+          <t>https://m.place.naver.com/place/1049963433</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -752,29 +748,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>지니네일</t>
+          <t>이뽐뷰티 강화점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>goto_seoul@naver.com</t>
+          <t>leebbom_kh@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1316-6480</t>
+          <t>0507-1385-2307</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 남문안길32번길 8 2층</t>
+          <t>인천광역시 강화군 강화읍 동문안길 7 B동 101호</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>http://www.instagram.com/jineenail</t>
+          <t>https://blog.naver.com/leebbom_kh</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -789,7 +785,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -809,13 +805,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="R4" t="n">
-        <v>4</v>
+        <v>115</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -824,17 +820,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1155579596</t>
+          <t>1404657024</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1155579596</t>
+          <t>https://m.place.naver.com/place/1404657024</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -846,34 +842,34 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>미뇽네일</t>
+          <t>비너스네일앤뷰티</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>akstjd1018@naver.com</t>
+          <t>hankyuldata@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1381-9702</t>
+          <t>0507-1309-4148</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 347-1 101호</t>
+          <t>인천광역시 강화군 강화읍 신문길 42 2층</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>http://pf.kakao.com/_hkxiqG</t>
+          <t>https://www.instagram.com/venus_nail4148</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -894,7 +890,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -903,13 +899,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>125</v>
+        <v>24</v>
       </c>
       <c r="Q5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>128</v>
+        <v>24</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -918,17 +914,17 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1280952259</t>
+          <t>1141156599</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1280952259</t>
+          <t>https://m.place.naver.com/place/1141156599</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -940,25 +936,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>코코로네일</t>
+          <t>레푸스 강화점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>romina97@naver.com</t>
+          <t>refuss_ganghwa@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0507-1409-2278</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 길상면 온수길 46</t>
+          <t>인천광역시 강화군 강화읍 충렬사로 25 남산빌딩 2층 202호</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.youtube.com/@강화레푸스</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -968,12 +968,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -989,17 +989,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1008,17 +1008,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1049963433</t>
+          <t>1506333714</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1049963433</t>
+          <t>https://m.place.naver.com/place/1506333714</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1030,25 +1030,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>네일하우스</t>
+          <t>네일홀릭</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>toy_21c@naver.com</t>
+          <t>minmin0319@naver.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0507-1480-4549</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 청하동길 12 1층</t>
+          <t>인천광역시 강화군 강화읍 강화대로 421 2층네일홀릭</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>http://Instagram.com/nail_house7930</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1058,7 +1062,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1083,13 +1087,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1098,17 +1102,17 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>37934661</t>
+          <t>1716746742</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/37934661</t>
+          <t>https://m.place.naver.com/place/1716746742</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1120,29 +1124,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>이뽐뷰티 강화점</t>
+          <t>퍼플리네일</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>leebbom_kh@naver.com</t>
+          <t>u_un0709@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0507-1385-2307</t>
+          <t>0507-1315-4140</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 동문안길 7 B동 101호</t>
+          <t>인천광역시 강화군 선원면 중앙로 162-3 2층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/leebbom_kh</t>
+          <t>https://www.instagram.com/purply._.nail/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1157,7 +1161,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1177,13 +1181,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="Q8" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>115</v>
+        <v>41</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1192,17 +1196,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1404657024</t>
+          <t>2094549338</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1404657024</t>
+          <t>https://m.place.naver.com/place/2094549338</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1214,29 +1218,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>뉴얼리네일</t>
+          <t>소소네일</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kimaechin01@naver.com</t>
+          <t>iamkimz@naver.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0507-1429-1729</t>
+          <t>0507-1327-9628</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 선원면 중앙로 162-31 서희스타힐스 106동 1층 상가</t>
+          <t>인천광역시 강화군 강화읍 강화대로404번길 9 2층 윈썸헤어&amp;소소네일</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/nurely_nail</t>
+          <t>https://www.instagram.com/sosonail_y?igsh=djM3NzVmbHM5eDRo&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1271,13 +1275,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1286,17 +1290,17 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2009541921</t>
+          <t>1958174820</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2009541921</t>
+          <t>https://m.place.naver.com/place/1958174820</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1308,29 +1312,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>비너스네일앤뷰티</t>
+          <t>온리원네일</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>hankyuldata@naver.com</t>
+          <t>nail_one@naver.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0507-1309-4148</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 신문길 42 2층</t>
+          <t>인천광역시 강화군 강화읍 강화대로248번길 28-4 1층 102호</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/venus_nail4148</t>
+          <t>https://www.instagram.com/__only_one__nail</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1365,13 +1365,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1380,17 +1380,17 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1141156599</t>
+          <t>2039624196</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1141156599</t>
+          <t>https://m.place.naver.com/place/2039624196</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1402,29 +1402,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>그레이스네일</t>
+          <t>무</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>lumirode@naver.com</t>
+          <t>sooks_room@naver.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0507-1379-5084</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로248번길 24 갑룡프라자 2층</t>
+          <t>인천광역시 강화군 강화읍 강화대로 394</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/grace_nail_?igsh=eGhhYXZlaGl0Z3hh&amp;utm_source=qr</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1434,7 +1430,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1455,17 +1451,17 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>159</v>
+        <v>5</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R11" t="n">
-        <v>160</v>
+        <v>8</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1474,17 +1470,17 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1030374689</t>
+          <t>36721147</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1030374689</t>
+          <t>https://m.place.naver.com/place/36721147</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1496,29 +1492,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>소소네일</t>
+          <t>뉴얼리네일</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>iamkimz@naver.com</t>
+          <t>kimaechin01@naver.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0507-1327-9628</t>
+          <t>0507-1429-1729</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로404번길 9 2층 윈썸헤어&amp;소소네일</t>
+          <t>인천광역시 강화군 선원면 중앙로 162-31 서희스타힐스 106동 1층 상가</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/sosonail_y?igsh=djM3NzVmbHM5eDRo&amp;utm_source=qr</t>
+          <t>https://www.instagram.com/nurely_nail</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1553,13 +1549,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="R12" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1568,17 +1564,17 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1958174820</t>
+          <t>2009541921</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1958174820</t>
+          <t>https://m.place.naver.com/place/2009541921</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1590,25 +1586,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>프프네일</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sooks_room@naver.com</t>
+          <t>daonnail0305@naver.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0507-1407-8841</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 394</t>
+          <t>인천광역시 강화군 강화읍 남문안길 5-1 1층</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/ff__nail</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1639,17 +1639,17 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P13" t="n">
         <v>5</v>
       </c>
       <c r="Q13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R13" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1658,17 +1658,17 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>36721147</t>
+          <t>1170338521</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/36721147</t>
+          <t>https://m.place.naver.com/place/1170338521</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1774,29 +1774,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>리네일아트 강화점</t>
+          <t>달빛네일</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>sg20092@naver.com</t>
+          <t>youwool1004@naver.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0507-1416-0155</t>
+          <t>0507-1316-8875</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 갑룡길 33-1</t>
+          <t>인천광역시 강화군 강화읍 강화대로 310 201호 달빛네일</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/sg20092</t>
+          <t>https://open.kakao.com/o/sLs1Sagi</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1822,22 +1822,22 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1846,17 +1846,17 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1180020313</t>
+          <t>2052753261</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1180020313</t>
+          <t>https://m.place.naver.com/place/2052753261</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1868,29 +1868,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>네일홀릭</t>
+          <t>제이네일</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>minmin0319@naver.com</t>
+          <t>morningapple6@naver.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>0507-1480-4549</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 421 2층네일홀릭</t>
+          <t>인천광역시 강화군 강화읍 향나무길28번길 13-1</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/j.nail_shop</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1900,7 +1896,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1921,14 +1917,14 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R16" t="n">
         <v>7</v>
@@ -1940,17 +1936,17 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1716746742</t>
+          <t>1237271418</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1716746742</t>
+          <t>https://m.place.naver.com/place/1237271418</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1962,29 +1958,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>퍼플리네일</t>
+          <t>지니네일</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>u_un0709@naver.com</t>
+          <t>goto_seoul@naver.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0507-1315-4140</t>
+          <t>0507-1316-6480</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 선원면 중앙로 162-3 2층</t>
+          <t>인천광역시 강화군 강화읍 남문안길32번길 8 2층</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/purply._.nail/</t>
+          <t>http://www.instagram.com/jineenail</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2019,13 +2015,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R17" t="n">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2034,17 +2030,17 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2094549338</t>
+          <t>1155579596</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2094549338</t>
+          <t>https://m.place.naver.com/place/1155579596</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2056,12 +2052,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>온리원네일</t>
+          <t>네일하우스</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>nail_one@naver.com</t>
+          <t>toy_21c@naver.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -2069,12 +2065,12 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로248번길 28-4 1층 102호</t>
+          <t>인천광역시 강화군 강화읍 청하동길 12 1층</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/__only_one__nail</t>
+          <t>http://Instagram.com/nail_house7930</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2105,18 +2101,18 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P18" t="n">
         <v>1</v>
       </c>
       <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
         <v>1</v>
       </c>
-      <c r="R18" t="n">
-        <v>2</v>
-      </c>
       <c r="S18" t="inlineStr">
         <is>
           <t>X</t>
@@ -2124,17 +2120,17 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2039624196</t>
+          <t>37934661</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2039624196</t>
+          <t>https://m.place.naver.com/place/37934661</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2146,29 +2142,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>레푸스 강화점</t>
+          <t>오니네일</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>refuss_ganghwa@naver.com</t>
+          <t>wjsska1907@naver.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0507-1409-2278</t>
+          <t>0507-1311-0663</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 충렬사로 25 남산빌딩 2층 202호</t>
+          <t>인천광역시 강화군 강화읍 갑룡길 29 1층, 카페88 내부위치</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@강화레푸스</t>
+          <t>http://instagram.com/oninail_</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2183,7 +2179,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2203,13 +2199,13 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R19" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2218,17 +2214,17 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1506333714</t>
+          <t>1245994155</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1506333714</t>
+          <t>https://m.place.naver.com/place/1245994155</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2240,25 +2236,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>제이네일</t>
+          <t>그레이스네일</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>morningapple6@naver.com</t>
+          <t>smsy7784@naver.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0507-1379-5084</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 향나무길28번길 13-1</t>
+          <t>인천광역시 강화군 강화읍 강화대로248번길 24 갑룡프라자 2층</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/j.nail_shop</t>
+          <t>https://www.instagram.com/grace_nail_?igsh=eGhhYXZlaGl0Z3hh&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2293,13 +2293,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>5</v>
+        <v>159</v>
       </c>
       <c r="Q20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" t="n">
-        <v>7</v>
+        <v>160</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2308,17 +2308,17 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1237271418</t>
+          <t>1030374689</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1237271418</t>
+          <t>https://m.place.naver.com/place/1030374689</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2330,34 +2330,34 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>달빛네일</t>
+          <t>미뇽네일</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>duoshan_sz@naver.com</t>
+          <t>akstjd1018@naver.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0507-1316-8875</t>
+          <t>0507-1381-9702</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로 310 201호 달빛네일</t>
+          <t>인천광역시 강화군 강화읍 강화대로 347-1 101호</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://open.kakao.com/o/sLs1Sagi</t>
+          <t>http://pf.kakao.com/_hkxiqG</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2387,13 +2387,13 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>2</v>
+        <v>125</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>2</v>
+        <v>128</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2402,17 +2402,17 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2052753261</t>
+          <t>1280952259</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2052753261</t>
+          <t>https://m.place.naver.com/place/1280952259</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>

</xml_diff>